<commit_message>
feat: Create a working version of the NHL odds analysis tool
This commit captures a functional state of the project before undergoing a refactoring to improve efficiency. It includes the core Python scripts for fetching data, running analysis, and managing the database.

- Add GEMINI.md for project context.
- Add a .gitignore file to exclude generated data, logs, and other artifacts.
- Save modifications to the main application logic and shell script.
</commit_message>
<xml_diff>
--- a/daily_odds/modelled_likelihoods_weight4_tenthOppositionFactor_2024-12-02.xlsx
+++ b/daily_odds/modelled_likelihoods_weight4_tenthOppositionFactor_2024-12-02.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10312"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexmann/Documents/Code_Learning/nhl_fromscratch/daily_odds/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:40009_{4B16D7FA-3AD2-AE4A-9B9D-3443AF83F18B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9973AB1A-B5A4-F34F-B358-BE31C798D4DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19760"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="modelled_likelihoods_weight4_te" sheetId="1" r:id="rId1"/>
@@ -248,7 +248,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="0.0%"/>
@@ -855,43 +855,43 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:S85" totalsRowShown="0">
-  <autoFilter ref="A1:S85"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:S85" totalsRowShown="0">
+  <autoFilter ref="A1:S85" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:S85">
     <sortCondition descending="1" ref="K1:K85"/>
   </sortState>
   <tableColumns count="19">
-    <tableColumn id="1" name="id"/>
-    <tableColumn id="2" name="player_name"/>
-    <tableColumn id="3" name="date" dataDxfId="10"/>
-    <tableColumn id="4" name="over_under"/>
-    <tableColumn id="5" name="points"/>
-    <tableColumn id="6" name="implied_likelihood" dataDxfId="9" dataCellStyle="Percent"/>
-    <tableColumn id="7" name="normal_likelihood" dataDxfId="8" dataCellStyle="Percent"/>
-    <tableColumn id="8" name="poisson_likelihood" dataDxfId="7" dataCellStyle="Percent"/>
-    <tableColumn id="9" name="raw_data_likelihood" dataDxfId="6" dataCellStyle="Percent"/>
-    <tableColumn id="10" name="weighted_likelihood" dataDxfId="5" dataCellStyle="Percent"/>
-    <tableColumn id="11" name="poisson_kelly" dataDxfId="4" dataCellStyle="Percent"/>
-    <tableColumn id="12" name="365 implied" dataDxfId="1" dataCellStyle="Percent">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="id"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="player_name"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="date" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="over_under"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="points"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="implied_likelihood" dataDxfId="9" dataCellStyle="Percent"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="normal_likelihood" dataDxfId="8" dataCellStyle="Percent"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="poisson_likelihood" dataDxfId="7" dataCellStyle="Percent"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="raw_data_likelihood" dataDxfId="6" dataCellStyle="Percent"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="weighted_likelihood" dataDxfId="5" dataCellStyle="Percent"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="poisson_kelly" dataDxfId="4" dataCellStyle="Percent"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="365 implied" dataDxfId="3" dataCellStyle="Percent">
       <calculatedColumnFormula>1/1.62</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" name="kelly/4 365" dataDxfId="3" dataCellStyle="Percent">
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="kelly/4 365" dataDxfId="2" dataCellStyle="Percent">
       <calculatedColumnFormula>(Table1[[#This Row],[poisson_likelihood]] - (1-Table1[[#This Row],[poisson_likelihood]])/(1/Table1[[#This Row],[365 implied]]-1))/4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" name="bet" dataCellStyle="Currency">
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="bet" dataCellStyle="Currency">
       <calculatedColumnFormula>Table1[[#This Row],[kelly/4 365]]*$W$2*$U$2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" name="99/pinn implied" dataDxfId="0" dataCellStyle="Percent">
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="99/pinn implied" dataDxfId="1" dataCellStyle="Percent">
       <calculatedColumnFormula>1/1.62</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" name="kelly/4 99" dataDxfId="2" dataCellStyle="Percent">
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="kelly/4 99" dataDxfId="0" dataCellStyle="Percent">
       <calculatedColumnFormula>(Table1[[#This Row],[poisson_likelihood]] - (1-Table1[[#This Row],[poisson_likelihood]])/(1/Table1[[#This Row],[99/pinn implied]]-1))/4</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" name="bet99/pinn" dataCellStyle="Currency">
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="bet99/pinn" dataCellStyle="Currency">
       <calculatedColumnFormula>Table1[[#This Row],[kelly/4 99]]*$W$2*$U$2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="18" name="W/L:"/>
-    <tableColumn id="19" name="del$" dataCellStyle="Currency">
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="W/L:"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="del$" dataCellStyle="Currency">
       <calculatedColumnFormula>IF(Table1[[#This Row],[W/L:]]="W", IF(Table1[[#This Row],[bet]]&gt;Table1[[#This Row],[bet99/pinn]],Table1[[#This Row],[bet]]*(1/Table1[[#This Row],[365 implied]])-Table1[[#This Row],[bet]],Table1[[#This Row],[bet99/pinn]]*(1/Table1[[#This Row],[99/pinn implied]])-Table1[[#This Row],[bet99/pinn]]), IF(Table1[[#This Row],[W/L:]]="L", IF(Table1[[#This Row],[bet]]&gt;Table1[[#This Row],[bet99/pinn]], -1*Table1[[#This Row],[bet]], -1*Table1[[#This Row],[bet99/pinn]]), 0))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1195,7 +1195,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Y85"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
@@ -1326,7 +1326,7 @@
         <v>7.0717161574111106E-2</v>
       </c>
       <c r="L2" s="2">
-        <f t="shared" ref="L2:L33" si="0">1/1.62</f>
+        <f t="shared" ref="L2" si="0">1/1.62</f>
         <v>0.61728395061728392</v>
       </c>
       <c r="M2" s="2">
@@ -1338,7 +1338,7 @@
         <v>124.37324062690509</v>
       </c>
       <c r="O2" s="2">
-        <f t="shared" ref="O2:O33" si="1">1/1.62</f>
+        <f t="shared" ref="O2" si="1">1/1.62</f>
         <v>0.61728395061728392</v>
       </c>
       <c r="P2" s="2">

</xml_diff>